<commit_message>
Updates because of mute with PTT
</commit_message>
<xml_diff>
--- a/Bill_of_Material.xlsx
+++ b/Bill_of_Material.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dirk/Libelle/OpenVario/e-Vario/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dirk/Libelle/OpenVario/e-Vario/Instructions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FBA9F5-E750-3F49-8A08-2DE269E6D56B}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9E11AE-5B96-6347-935F-DF51BA844D54}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="15540" xr2:uid="{A71850B3-3A10-CA42-999C-A02A84AA5A96}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="162">
   <si>
     <t>Value</t>
   </si>
@@ -163,9 +163,6 @@
   </si>
   <si>
     <t>NCP 1117 ST33T3G </t>
-  </si>
-  <si>
-    <t>JST XH2P BU</t>
   </si>
   <si>
     <t>﻿STF-WOELBKLAPPEN</t>
@@ -510,9 +507,6 @@
   </si>
   <si>
     <t>JST - socket housing, 1x3-pin - XH</t>
-  </si>
-  <si>
-    <t>JST — socket housing, 1x2-pin - XH</t>
   </si>
   <si>
     <t>Toggle switch 6A-125VAC, 1x On-Off-ON</t>
@@ -1387,7 +1381,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1406,7 +1400,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1420,7 +1414,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
@@ -1437,10 +1431,10 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1449,7 +1443,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1463,10 +1457,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9" t="s">
         <v>94</v>
-      </c>
-      <c r="E9" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1488,7 +1482,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
@@ -1500,15 +1494,15 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="3">
         <v>2</v>
@@ -1517,16 +1511,16 @@
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C13" s="3">
         <v>1</v>
@@ -1535,16 +1529,16 @@
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -1553,16 +1547,16 @@
         <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
@@ -1571,16 +1565,16 @@
         <v>10</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" s="3">
         <v>1</v>
@@ -1589,16 +1583,16 @@
         <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C17" s="3">
         <v>1</v>
@@ -1607,13 +1601,13 @@
         <v>10</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
@@ -1630,10 +1624,10 @@
     </row>
     <row r="19" spans="1:6" s="3" customFormat="1">
       <c r="A19" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" s="3">
         <v>5</v>
@@ -1642,15 +1636,15 @@
         <v>10</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="3" customFormat="1">
       <c r="A20" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C20" s="3">
         <v>4</v>
@@ -1659,15 +1653,15 @@
         <v>10</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21">
         <v>5</v>
@@ -1681,10 +1675,10 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C22" s="3">
         <v>2</v>
@@ -1693,15 +1687,15 @@
         <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C23" s="3">
         <v>1</v>
@@ -1710,15 +1704,15 @@
         <v>10</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C24" s="3">
         <v>1</v>
@@ -1727,15 +1721,15 @@
         <v>10</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C25" s="3">
         <v>2</v>
@@ -1744,12 +1738,12 @@
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="4" customFormat="1">
       <c r="A26" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>23</v>
@@ -1763,10 +1757,10 @@
     </row>
     <row r="27" spans="1:6" s="4" customFormat="1">
       <c r="A27" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C27" s="3">
         <v>1</v>
@@ -1775,7 +1769,7 @@
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F27" s="3"/>
     </row>
@@ -1784,7 +1778,7 @@
         <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1798,7 +1792,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
@@ -1810,12 +1804,12 @@
         <v>10</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
@@ -1824,7 +1818,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E30" s="3"/>
     </row>
@@ -1854,10 +1848,10 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35">
         <v>4</v>
@@ -1871,10 +1865,10 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C36" s="3">
         <v>1</v>
@@ -1883,16 +1877,16 @@
         <v>10</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F36" s="3"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1906,7 +1900,7 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
         <v>29</v>
@@ -1919,10 +1913,10 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C39" s="9">
         <v>1</v>
@@ -1933,41 +1927,41 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B40" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" t="s">
         <v>47</v>
-      </c>
-      <c r="C40">
-        <v>1</v>
-      </c>
-      <c r="D40" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1">
       <c r="A41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B41" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s">
         <v>92</v>
-      </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-      <c r="D41" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B42" t="s">
         <v>8</v>
@@ -1984,7 +1978,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B43" t="s">
         <v>30</v>
@@ -2001,7 +1995,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B44" t="s">
         <v>30</v>
@@ -2013,15 +2007,15 @@
         <v>10</v>
       </c>
       <c r="E44" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:6">
-      <c r="A45" t="s">
-        <v>143</v>
+      <c r="A45" s="3" t="s">
+        <v>141</v>
       </c>
       <c r="B45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2030,15 +2024,15 @@
         <v>10</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2047,15 +2041,15 @@
         <v>10</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C47">
         <v>2</v>
@@ -2069,7 +2063,7 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B48" t="s">
         <v>15</v>
@@ -2078,7 +2072,7 @@
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E48" s="3"/>
     </row>
@@ -2098,7 +2092,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B52" t="s">
         <v>33</v>
@@ -2110,12 +2104,12 @@
         <v>10</v>
       </c>
       <c r="E52" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -2132,7 +2126,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>19</v>
@@ -2149,7 +2143,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B55" t="s">
         <v>19</v>
@@ -2166,7 +2160,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B56" t="s">
         <v>19</v>
@@ -2183,7 +2177,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -2197,7 +2191,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B58" t="s">
         <v>36</v>
@@ -2206,12 +2200,12 @@
         <v>1</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C59">
         <v>2</v>
@@ -2220,7 +2214,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C60">
         <v>2</v>
@@ -2229,12 +2223,12 @@
         <v>37</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C61">
         <v>2</v>
@@ -2318,16 +2312,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2338,24 +2332,24 @@
         <v>17</v>
       </c>
       <c r="C2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>66</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2363,97 +2357,97 @@
         <v>26</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2461,13 +2455,13 @@
         <v>44</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2510,16 +2504,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2527,27 +2521,27 @@
         <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2625,16 +2619,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2642,27 +2636,27 @@
         <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4">

</xml_diff>